<commit_message>
chore:data update Binance USDT perpetual data files
</commit_message>
<xml_diff>
--- a/records/weeks/2026-03-09_2026-03-15/2026-03-15.xlsx
+++ b/records/weeks/2026-03-09_2026-03-15/2026-03-15.xlsx
@@ -535,7 +535,7 @@
         <v>71429</v>
       </c>
       <c r="K2" s="1" t="n">
-        <v>71481.2</v>
+        <v>71457.60000000001</v>
       </c>
       <c r="L2" s="1" t="n">
         <v>71675.60000000001</v>
@@ -578,7 +578,7 @@
         <v>2092.15</v>
       </c>
       <c r="K3" s="1" t="n">
-        <v>2092.01</v>
+        <v>2091.4</v>
       </c>
       <c r="L3" s="1" t="n">
         <v>2115.97</v>
@@ -621,7 +621,7 @@
         <v>87.68000000000001</v>
       </c>
       <c r="K4" s="1" t="n">
-        <v>87.87</v>
+        <v>87.83</v>
       </c>
       <c r="L4" s="1" t="n">
         <v>88.37</v>
@@ -664,7 +664,7 @@
         <v>3.959</v>
       </c>
       <c r="K5" s="1" t="n">
-        <v>3.957</v>
+        <v>3.959</v>
       </c>
       <c r="L5" s="1" t="n">
         <v>4.025</v>
@@ -707,7 +707,7 @@
         <v>0.09522</v>
       </c>
       <c r="K6" s="1" t="n">
-        <v>0.09544</v>
+        <v>0.09537</v>
       </c>
       <c r="L6" s="1" t="n">
         <v>0.09632</v>
@@ -750,13 +750,13 @@
         <v>1.4177</v>
       </c>
       <c r="K7" s="1" t="n">
-        <v>1.4148</v>
+        <v>1.4143</v>
       </c>
       <c r="L7" s="1" t="n">
         <v>1.4234</v>
       </c>
       <c r="M7" s="1" t="n">
-        <v>1.4148</v>
+        <v>1.4143</v>
       </c>
     </row>
     <row r="8">
@@ -793,7 +793,7 @@
         <v>23.678</v>
       </c>
       <c r="K8" s="1" t="n">
-        <v>23.796</v>
+        <v>23.799</v>
       </c>
       <c r="L8" s="1" t="n">
         <v>24.384</v>
@@ -879,13 +879,13 @@
         <v>0.009865000000000001</v>
       </c>
       <c r="K10" s="1" t="n">
-        <v>0.009819</v>
+        <v>0.009821</v>
       </c>
       <c r="L10" s="1" t="n">
         <v>0.010135</v>
       </c>
       <c r="M10" s="1" t="n">
-        <v>0.009819</v>
+        <v>0.009821</v>
       </c>
     </row>
     <row r="11">
@@ -922,7 +922,7 @@
         <v>0.09208</v>
       </c>
       <c r="K11" s="1" t="n">
-        <v>0.09291000000000001</v>
+        <v>0.09313</v>
       </c>
       <c r="L11" s="1" t="n">
         <v>0.09659</v>
@@ -965,13 +965,13 @@
         <v>0.011676</v>
       </c>
       <c r="K12" s="1" t="n">
-        <v>0.011554</v>
+        <v>0.011543</v>
       </c>
       <c r="L12" s="1" t="n">
         <v>0.011737</v>
       </c>
       <c r="M12" s="1" t="n">
-        <v>0.011554</v>
+        <v>0.011543</v>
       </c>
     </row>
     <row r="13">
@@ -1008,7 +1008,7 @@
         <v>37.335</v>
       </c>
       <c r="K13" s="1" t="n">
-        <v>37.392</v>
+        <v>37.373</v>
       </c>
       <c r="L13" s="1" t="n">
         <v>37.523</v>
@@ -1051,7 +1051,7 @@
         <v>659.41</v>
       </c>
       <c r="K14" s="1" t="n">
-        <v>659.95</v>
+        <v>659.66</v>
       </c>
       <c r="L14" s="1" t="n">
         <v>661.97</v>
@@ -1094,7 +1094,7 @@
         <v>227.19</v>
       </c>
       <c r="K15" s="1" t="n">
-        <v>227.98</v>
+        <v>227.83</v>
       </c>
       <c r="L15" s="1" t="n">
         <v>228.05</v>
@@ -1137,7 +1137,7 @@
         <v>0.003351</v>
       </c>
       <c r="K16" s="1" t="n">
-        <v>0.0033583</v>
+        <v>0.003356</v>
       </c>
       <c r="L16" s="1" t="n">
         <v>0.0033804</v>
@@ -1223,7 +1223,7 @@
         <v>1.0001</v>
       </c>
       <c r="K18" s="1" t="n">
-        <v>1.0014</v>
+        <v>1.0012</v>
       </c>
       <c r="L18" s="1" t="n">
         <v>1.005</v>
@@ -1266,13 +1266,13 @@
         <v>0.8915</v>
       </c>
       <c r="K19" s="1" t="n">
-        <v>0.887</v>
+        <v>0.8859</v>
       </c>
       <c r="L19" s="1" t="n">
         <v>0.9177999999999999</v>
       </c>
       <c r="M19" s="1" t="n">
-        <v>0.8867</v>
+        <v>0.8859</v>
       </c>
     </row>
     <row r="20">
@@ -1309,7 +1309,7 @@
         <v>0.2634</v>
       </c>
       <c r="K20" s="1" t="n">
-        <v>0.2635</v>
+        <v>0.2633</v>
       </c>
       <c r="L20" s="1" t="n">
         <v>0.2657</v>
@@ -1352,7 +1352,7 @@
         <v>0.57885</v>
       </c>
       <c r="K21" s="1" t="n">
-        <v>0.57779</v>
+        <v>0.57803</v>
       </c>
       <c r="L21" s="1" t="n">
         <v>0.59453</v>
@@ -1395,7 +1395,7 @@
         <v>9.151999999999999</v>
       </c>
       <c r="K22" s="1" t="n">
-        <v>9.163</v>
+        <v>9.157</v>
       </c>
       <c r="L22" s="1" t="n">
         <v>9.257999999999999</v>
@@ -1481,7 +1481,7 @@
         <v>9.728</v>
       </c>
       <c r="K24" s="1" t="n">
-        <v>9.738</v>
+        <v>9.731</v>
       </c>
       <c r="L24" s="1" t="n">
         <v>9.853999999999999</v>
@@ -1567,10 +1567,10 @@
         <v>0.06913999999999999</v>
       </c>
       <c r="K26" s="1" t="n">
-        <v>0.06951</v>
+        <v>0.06956</v>
       </c>
       <c r="L26" s="1" t="n">
-        <v>0.06951</v>
+        <v>0.06956</v>
       </c>
       <c r="M26" s="1" t="n">
         <v>0.06789000000000001</v>
@@ -1610,7 +1610,7 @@
         <v>1.417</v>
       </c>
       <c r="K27" s="1" t="n">
-        <v>1.418</v>
+        <v>1.417</v>
       </c>
       <c r="L27" s="1" t="n">
         <v>1.437</v>
@@ -1653,13 +1653,13 @@
         <v>1.332</v>
       </c>
       <c r="K28" s="1" t="n">
-        <v>1.331</v>
+        <v>1.33</v>
       </c>
       <c r="L28" s="1" t="n">
         <v>1.357</v>
       </c>
       <c r="M28" s="1" t="n">
-        <v>1.331</v>
+        <v>1.33</v>
       </c>
     </row>
     <row r="29">
@@ -1739,7 +1739,7 @@
         <v>1.2196</v>
       </c>
       <c r="K30" s="1" t="n">
-        <v>1.2226</v>
+        <v>1.2222</v>
       </c>
       <c r="L30" s="1" t="n">
         <v>1.2415</v>
@@ -1825,7 +1825,7 @@
         <v>0.888</v>
       </c>
       <c r="K32" s="1" t="n">
-        <v>0.888</v>
+        <v>0.887</v>
       </c>
       <c r="L32" s="1" t="n">
         <v>0.892</v>
@@ -1868,7 +1868,7 @@
         <v>0.001964</v>
       </c>
       <c r="K33" s="1" t="n">
-        <v>0.001976</v>
+        <v>0.001975</v>
       </c>
       <c r="L33" s="1" t="n">
         <v>0.00201</v>
@@ -1911,7 +1911,7 @@
         <v>0.15848</v>
       </c>
       <c r="K34" s="1" t="n">
-        <v>0.17297</v>
+        <v>0.17154</v>
       </c>
       <c r="L34" s="1" t="n">
         <v>0.18819</v>
@@ -2040,7 +2040,7 @@
         <v>112.63</v>
       </c>
       <c r="K37" s="1" t="n">
-        <v>112.61</v>
+        <v>112.52</v>
       </c>
       <c r="L37" s="1" t="n">
         <v>113.73</v>
@@ -2083,7 +2083,7 @@
         <v>0.21767</v>
       </c>
       <c r="K38" s="1" t="n">
-        <v>0.21802</v>
+        <v>0.21801</v>
       </c>
       <c r="L38" s="1" t="n">
         <v>0.21948</v>
@@ -2169,13 +2169,13 @@
         <v>0.36604</v>
       </c>
       <c r="K40" s="1" t="n">
-        <v>0.36222</v>
+        <v>0.36364</v>
       </c>
       <c r="L40" s="1" t="n">
         <v>0.37243</v>
       </c>
       <c r="M40" s="1" t="n">
-        <v>0.36222</v>
+        <v>0.36364</v>
       </c>
     </row>
     <row r="41">
@@ -2212,7 +2212,7 @@
         <v>55.19</v>
       </c>
       <c r="K41" s="1" t="n">
-        <v>55.2</v>
+        <v>55.18</v>
       </c>
       <c r="L41" s="1" t="n">
         <v>55.39</v>
@@ -2255,7 +2255,7 @@
         <v>0.0010896</v>
       </c>
       <c r="K42" s="1" t="n">
-        <v>0.0010906</v>
+        <v>0.0010897</v>
       </c>
       <c r="L42" s="1" t="n">
         <v>0.0011009</v>
@@ -2341,10 +2341,10 @@
         <v>0.6514</v>
       </c>
       <c r="K44" s="1" t="n">
-        <v>0.6542</v>
+        <v>0.6539</v>
       </c>
       <c r="L44" s="1" t="n">
-        <v>0.6542</v>
+        <v>0.6539</v>
       </c>
       <c r="M44" s="1" t="n">
         <v>0.6421</v>
@@ -2384,7 +2384,7 @@
         <v>0.3573</v>
       </c>
       <c r="K45" s="1" t="n">
-        <v>0.3582</v>
+        <v>0.3579</v>
       </c>
       <c r="L45" s="1" t="n">
         <v>0.3612</v>
@@ -2427,7 +2427,7 @@
         <v>0.03222</v>
       </c>
       <c r="K46" s="1" t="n">
-        <v>0.03231</v>
+        <v>0.03229</v>
       </c>
       <c r="L46" s="1" t="n">
         <v>0.03257</v>
@@ -2470,10 +2470,10 @@
         <v>0.06630999999999999</v>
       </c>
       <c r="K47" s="1" t="n">
-        <v>0.06691</v>
+        <v>0.06683</v>
       </c>
       <c r="L47" s="1" t="n">
-        <v>0.06691</v>
+        <v>0.06689000000000001</v>
       </c>
       <c r="M47" s="1" t="n">
         <v>0.06568</v>
@@ -2513,7 +2513,7 @@
         <v>0.7127</v>
       </c>
       <c r="K48" s="1" t="n">
-        <v>0.715</v>
+        <v>0.7149</v>
       </c>
       <c r="L48" s="1" t="n">
         <v>0.7189</v>
@@ -2556,7 +2556,7 @@
         <v>0.004117</v>
       </c>
       <c r="K49" s="1" t="n">
-        <v>0.004084</v>
+        <v>0.004086</v>
       </c>
       <c r="L49" s="1" t="n">
         <v>0.004215</v>
@@ -2642,7 +2642,7 @@
         <v>0.04011</v>
       </c>
       <c r="K51" s="1" t="n">
-        <v>0.04018</v>
+        <v>0.04019</v>
       </c>
       <c r="L51" s="1" t="n">
         <v>0.04045</v>
@@ -2685,7 +2685,7 @@
         <v>0.1661</v>
       </c>
       <c r="K52" s="1" t="n">
-        <v>0.1668</v>
+        <v>0.1667</v>
       </c>
       <c r="L52" s="1" t="n">
         <v>0.1672</v>
@@ -2728,7 +2728,7 @@
         <v>0.01817</v>
       </c>
       <c r="K53" s="1" t="n">
-        <v>0.01805</v>
+        <v>0.01803</v>
       </c>
       <c r="L53" s="1" t="n">
         <v>0.01825</v>
@@ -2771,7 +2771,7 @@
         <v>0.007299</v>
       </c>
       <c r="K54" s="1" t="n">
-        <v>0.007325</v>
+        <v>0.007317</v>
       </c>
       <c r="L54" s="1" t="n">
         <v>0.007365</v>
@@ -2814,7 +2814,7 @@
         <v>3.95</v>
       </c>
       <c r="K55" s="1" t="n">
-        <v>3.958</v>
+        <v>3.957</v>
       </c>
       <c r="L55" s="1" t="n">
         <v>3.985</v>
@@ -2857,13 +2857,13 @@
         <v>0.016453</v>
       </c>
       <c r="K56" s="1" t="n">
-        <v>0.01637</v>
+        <v>0.016361</v>
       </c>
       <c r="L56" s="1" t="n">
         <v>0.016649</v>
       </c>
       <c r="M56" s="1" t="n">
-        <v>0.016367</v>
+        <v>0.016361</v>
       </c>
     </row>
     <row r="57">
@@ -2900,7 +2900,7 @@
         <v>0.1073</v>
       </c>
       <c r="K57" s="1" t="n">
-        <v>0.1079</v>
+        <v>0.1078</v>
       </c>
       <c r="L57" s="1" t="n">
         <v>0.1092</v>
@@ -3029,7 +3029,7 @@
         <v>0.005841</v>
       </c>
       <c r="K60" s="1" t="n">
-        <v>0.005851</v>
+        <v>0.005848</v>
       </c>
       <c r="L60" s="1" t="n">
         <v>0.005861</v>
@@ -3072,7 +3072,7 @@
         <v>0.09515999999999999</v>
       </c>
       <c r="K61" s="1" t="n">
-        <v>0.09532</v>
+        <v>0.09525</v>
       </c>
       <c r="L61" s="1" t="n">
         <v>0.09576</v>
@@ -3115,7 +3115,7 @@
         <v>0.9212</v>
       </c>
       <c r="K62" s="1" t="n">
-        <v>0.9208</v>
+        <v>0.9201</v>
       </c>
       <c r="L62" s="1" t="n">
         <v>0.9330000000000001</v>
@@ -3244,13 +3244,13 @@
         <v>359.12</v>
       </c>
       <c r="K65" s="1" t="n">
-        <v>356.58</v>
+        <v>356.82</v>
       </c>
       <c r="L65" s="1" t="n">
         <v>359.12</v>
       </c>
       <c r="M65" s="1" t="n">
-        <v>356.58</v>
+        <v>356.82</v>
       </c>
     </row>
     <row r="66">
@@ -3330,7 +3330,7 @@
         <v>0.2344</v>
       </c>
       <c r="K67" s="1" t="n">
-        <v>0.2344</v>
+        <v>0.2343</v>
       </c>
       <c r="L67" s="1" t="n">
         <v>0.2346</v>
@@ -3416,13 +3416,13 @@
         <v>0.1941</v>
       </c>
       <c r="K69" s="1" t="n">
-        <v>0.1933</v>
+        <v>0.1931</v>
       </c>
       <c r="L69" s="1" t="n">
         <v>0.1995</v>
       </c>
       <c r="M69" s="1" t="n">
-        <v>0.1933</v>
+        <v>0.1931</v>
       </c>
     </row>
     <row r="70">
@@ -3459,7 +3459,7 @@
         <v>0.16746</v>
       </c>
       <c r="K70" s="1" t="n">
-        <v>0.16775</v>
+        <v>0.16766</v>
       </c>
       <c r="L70" s="1" t="n">
         <v>0.16813</v>
@@ -3545,7 +3545,7 @@
         <v>0.7265</v>
       </c>
       <c r="K72" s="1" t="n">
-        <v>0.7296</v>
+        <v>0.7288</v>
       </c>
       <c r="L72" s="1" t="n">
         <v>0.7361</v>
@@ -3588,7 +3588,7 @@
         <v>0.00842</v>
       </c>
       <c r="K73" s="1" t="n">
-        <v>0.008410000000000001</v>
+        <v>0.00842</v>
       </c>
       <c r="L73" s="1" t="n">
         <v>0.00851</v>
@@ -3631,7 +3631,7 @@
         <v>0.005935</v>
       </c>
       <c r="K74" s="1" t="n">
-        <v>0.005951</v>
+        <v>0.005947</v>
       </c>
       <c r="L74" s="1" t="n">
         <v>0.006009</v>
@@ -3717,7 +3717,7 @@
         <v>0.3127</v>
       </c>
       <c r="K76" s="1" t="n">
-        <v>0.3157</v>
+        <v>0.3156</v>
       </c>
       <c r="L76" s="1" t="n">
         <v>0.3167</v>
@@ -3760,7 +3760,7 @@
         <v>0.1016</v>
       </c>
       <c r="K77" s="1" t="n">
-        <v>0.1016</v>
+        <v>0.1015</v>
       </c>
       <c r="L77" s="1" t="n">
         <v>0.1031</v>
@@ -3846,7 +3846,7 @@
         <v>0.06736</v>
       </c>
       <c r="K79" s="1" t="n">
-        <v>0.06802</v>
+        <v>0.06798999999999999</v>
       </c>
       <c r="L79" s="1" t="n">
         <v>0.0689</v>
@@ -3975,7 +3975,7 @@
         <v>8.298</v>
       </c>
       <c r="K82" s="1" t="n">
-        <v>8.305999999999999</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="L82" s="1" t="n">
         <v>8.390000000000001</v>
@@ -4018,7 +4018,7 @@
         <v>0.0006535</v>
       </c>
       <c r="K83" s="1" t="n">
-        <v>0.0006533</v>
+        <v>0.0006528</v>
       </c>
       <c r="L83" s="1" t="n">
         <v>0.0006535</v>
@@ -4061,10 +4061,10 @@
         <v>0.4349</v>
       </c>
       <c r="K84" s="1" t="n">
-        <v>0.4383</v>
+        <v>0.4386</v>
       </c>
       <c r="L84" s="1" t="n">
-        <v>0.4383</v>
+        <v>0.4386</v>
       </c>
       <c r="M84" s="1" t="n">
         <v>0.4031</v>
@@ -4147,7 +4147,7 @@
         <v>0.05333</v>
       </c>
       <c r="K86" s="1" t="n">
-        <v>0.05336</v>
+        <v>0.05333</v>
       </c>
       <c r="L86" s="1" t="n">
         <v>0.05372</v>
@@ -4190,7 +4190,7 @@
         <v>0.00313</v>
       </c>
       <c r="K87" s="1" t="n">
-        <v>0.003145</v>
+        <v>0.003146</v>
       </c>
       <c r="L87" s="1" t="n">
         <v>0.003173</v>
@@ -4276,7 +4276,7 @@
         <v>0.02875</v>
       </c>
       <c r="K89" s="1" t="n">
-        <v>0.02844</v>
+        <v>0.0284</v>
       </c>
       <c r="L89" s="1" t="n">
         <v>0.02875</v>
@@ -4319,7 +4319,7 @@
         <v>0.3491</v>
       </c>
       <c r="K90" s="1" t="n">
-        <v>0.3496</v>
+        <v>0.3493</v>
       </c>
       <c r="L90" s="1" t="n">
         <v>0.3576</v>
@@ -4362,7 +4362,7 @@
         <v>0.08058999999999999</v>
       </c>
       <c r="K91" s="1" t="n">
-        <v>0.08035</v>
+        <v>0.08037999999999999</v>
       </c>
       <c r="L91" s="1" t="n">
         <v>0.08494</v>
@@ -4405,13 +4405,13 @@
         <v>0.4058</v>
       </c>
       <c r="K92" s="1" t="n">
-        <v>0.401</v>
+        <v>0.4011</v>
       </c>
       <c r="L92" s="1" t="n">
         <v>0.4413</v>
       </c>
       <c r="M92" s="1" t="n">
-        <v>0.401</v>
+        <v>0.4011</v>
       </c>
     </row>
     <row r="93">
@@ -4448,10 +4448,10 @@
         <v>2.0339</v>
       </c>
       <c r="K93" s="1" t="n">
-        <v>2.0572</v>
+        <v>2.0546</v>
       </c>
       <c r="L93" s="1" t="n">
-        <v>2.0572</v>
+        <v>2.0546</v>
       </c>
       <c r="M93" s="1" t="n">
         <v>2.0298</v>
@@ -4491,7 +4491,7 @@
         <v>0.2638</v>
       </c>
       <c r="K94" s="1" t="n">
-        <v>0.2644</v>
+        <v>0.2643</v>
       </c>
       <c r="L94" s="1" t="n">
         <v>0.2665</v>
@@ -4534,7 +4534,7 @@
         <v>0.04408</v>
       </c>
       <c r="K95" s="1" t="n">
-        <v>0.04394</v>
+        <v>0.04393</v>
       </c>
       <c r="L95" s="1" t="n">
         <v>0.04459</v>
@@ -4577,13 +4577,13 @@
         <v>0.005829</v>
       </c>
       <c r="K96" s="1" t="n">
-        <v>0.005811</v>
+        <v>0.005807</v>
       </c>
       <c r="L96" s="1" t="n">
         <v>0.006121</v>
       </c>
       <c r="M96" s="1" t="n">
-        <v>0.005811</v>
+        <v>0.005807</v>
       </c>
     </row>
     <row r="97">
@@ -4663,7 +4663,7 @@
         <v>5.147</v>
       </c>
       <c r="K98" s="1" t="n">
-        <v>5.169</v>
+        <v>5.173</v>
       </c>
       <c r="L98" s="1" t="n">
         <v>5.331</v>
@@ -4749,7 +4749,7 @@
         <v>0.5592</v>
       </c>
       <c r="K100" s="1" t="n">
-        <v>0.5594</v>
+        <v>0.5592</v>
       </c>
       <c r="L100" s="1" t="n">
         <v>0.5602</v>
@@ -4835,7 +4835,7 @@
         <v>33.3</v>
       </c>
       <c r="K102" s="1" t="n">
-        <v>33.34</v>
+        <v>33.33</v>
       </c>
       <c r="L102" s="1" t="n">
         <v>33.79</v>
@@ -4878,13 +4878,13 @@
         <v>0.03333</v>
       </c>
       <c r="K103" s="1" t="n">
-        <v>0.03318</v>
+        <v>0.03317</v>
       </c>
       <c r="L103" s="1" t="n">
         <v>0.03387</v>
       </c>
       <c r="M103" s="1" t="n">
-        <v>0.03318</v>
+        <v>0.03317</v>
       </c>
     </row>
     <row r="104">
@@ -4921,7 +4921,7 @@
         <v>0.06680999999999999</v>
       </c>
       <c r="K104" s="1" t="n">
-        <v>0.06695</v>
+        <v>0.06689000000000001</v>
       </c>
       <c r="L104" s="1" t="n">
         <v>0.06738</v>
@@ -4964,7 +4964,7 @@
         <v>1.2874</v>
       </c>
       <c r="K105" s="1" t="n">
-        <v>1.2877</v>
+        <v>1.2875</v>
       </c>
       <c r="L105" s="1" t="n">
         <v>1.2942</v>
@@ -5050,7 +5050,7 @@
         <v>0.119</v>
       </c>
       <c r="K107" s="1" t="n">
-        <v>0.12</v>
+        <v>0.119</v>
       </c>
       <c r="L107" s="1" t="n">
         <v>0.12</v>
@@ -5093,7 +5093,7 @@
         <v>0.09601999999999999</v>
       </c>
       <c r="K108" s="1" t="n">
-        <v>0.09608</v>
+        <v>0.09604</v>
       </c>
       <c r="L108" s="1" t="n">
         <v>0.09637</v>
@@ -5136,13 +5136,13 @@
         <v>0.13713</v>
       </c>
       <c r="K109" s="1" t="n">
-        <v>0.13611</v>
+        <v>0.13609</v>
       </c>
       <c r="L109" s="1" t="n">
         <v>0.14159</v>
       </c>
       <c r="M109" s="1" t="n">
-        <v>0.13611</v>
+        <v>0.13609</v>
       </c>
     </row>
     <row r="110">
@@ -5179,7 +5179,7 @@
         <v>5.954</v>
       </c>
       <c r="K110" s="1" t="n">
-        <v>6.008</v>
+        <v>6.002</v>
       </c>
       <c r="L110" s="1" t="n">
         <v>6.088</v>
@@ -5222,7 +5222,7 @@
         <v>1.087</v>
       </c>
       <c r="K111" s="1" t="n">
-        <v>1.091</v>
+        <v>1.09</v>
       </c>
       <c r="L111" s="1" t="n">
         <v>1.096</v>
@@ -5265,10 +5265,10 @@
         <v>0.029172</v>
       </c>
       <c r="K112" s="1" t="n">
-        <v>0.02929</v>
+        <v>0.029288</v>
       </c>
       <c r="L112" s="1" t="n">
-        <v>0.02929</v>
+        <v>0.029288</v>
       </c>
       <c r="M112" s="1" t="n">
         <v>0.028451</v>
@@ -5351,13 +5351,13 @@
         <v>0.0573</v>
       </c>
       <c r="K114" s="1" t="n">
-        <v>0.05693</v>
+        <v>0.05698</v>
       </c>
       <c r="L114" s="1" t="n">
         <v>0.05776</v>
       </c>
       <c r="M114" s="1" t="n">
-        <v>0.05693</v>
+        <v>0.05698</v>
       </c>
     </row>
     <row r="115">
@@ -5394,13 +5394,13 @@
         <v>0.12761</v>
       </c>
       <c r="K115" s="1" t="n">
-        <v>0.12715</v>
+        <v>0.12716</v>
       </c>
       <c r="L115" s="1" t="n">
         <v>0.12869</v>
       </c>
       <c r="M115" s="1" t="n">
-        <v>0.12715</v>
+        <v>0.12716</v>
       </c>
     </row>
     <row r="116">
@@ -5566,7 +5566,7 @@
         <v>0.04558</v>
       </c>
       <c r="K119" s="1" t="n">
-        <v>0.04553</v>
+        <v>0.04554</v>
       </c>
       <c r="L119" s="1" t="n">
         <v>0.04657</v>
@@ -5609,7 +5609,7 @@
         <v>3.058</v>
       </c>
       <c r="K120" s="1" t="n">
-        <v>3.065</v>
+        <v>3.063</v>
       </c>
       <c r="L120" s="1" t="n">
         <v>3.08</v>
@@ -5652,13 +5652,13 @@
         <v>0.3018</v>
       </c>
       <c r="K121" s="1" t="n">
-        <v>0.3018</v>
+        <v>0.3017</v>
       </c>
       <c r="L121" s="1" t="n">
         <v>0.3059</v>
       </c>
       <c r="M121" s="1" t="n">
-        <v>0.3018</v>
+        <v>0.3017</v>
       </c>
     </row>
     <row r="122">

</xml_diff>